<commit_message>
Rapport et cahier de recette des tests d'écran : 369 / 422 après la reprise des tests d'essai interrompu
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/recette/CAHIER_RECETTE_COMPLET_2026-10-30.xlsx
+++ b/docs/recette/CAHIER_RECETTE_COMPLET_2026-10-30.xlsx
@@ -653,7 +653,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>422 tests joués par l'écran, 366 OK, 56 en échec. Chaque test a été joué seul, par le vrai chemin de l'écran, et retire ses données à la fin.</t>
+          <t>422 tests joués par l'écran, 369 OK, 53 en échec. Chaque test a été joué seul, par le vrai chemin de l'écran, et retire ses données à la fin.</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>SYNTHÈSE — 422 tests, 366 OK, 56 en échec selon Claude</t>
+          <t>SYNTHÈSE — 422 tests, 369 OK, 53 en échec selon Claude</t>
         </is>
       </c>
     </row>
@@ -4128,10 +4128,10 @@
         <v>282</v>
       </c>
       <c r="D32" t="n">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="E32" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F32">
         <f>COUNTA('Retours des officines'!$I$5:$I$286)</f>
@@ -8833,7 +8833,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>282 tests : 242 OK, 40 en échec selon Claude</t>
+          <t>282 tests : 245 OK, 37 en échec selon Claude</t>
         </is>
       </c>
     </row>
@@ -11555,22 +11555,31 @@
 Tout ce que le test cree est retire (ventes, copies, annulations, mouvements, stock remis).</t>
         </is>
       </c>
-      <c r="D50" s="9" t="inlineStr"/>
-      <c r="E50" s="11" t="inlineStr">
-        <is>
-          <t>Échec</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="inlineStr">
-        <is>
-          <t>Test arrêté (code 1) avant la fin, sans contrôle en écart</t>
-        </is>
-      </c>
-      <c r="G50" s="9" t="inlineStr">
-        <is>
-          <t>Données d'essai : Clients d'essai restés en base après l'arrêt des serveurs à 11 h 07 (le test ne peut pas recréer son jeu d'essai) ; passait le matin. À rejouer après nettoyage.</t>
-        </is>
-      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>13 / 13 conformes
+✓ Précondition : vente de 2 produits clôturée en différé pour le client 1 [{"msg":"Opération effectuée avec success","ref":"5a7f60e8-129c-49e4-9dd4-e75cb9038075","success":true,"copy":false} e2e-dmod-c1|3580|3580|is_Closed]
+✓ Précondition : 1 produit réglé (reste = 1 produit) [{"msg":"Opération effectuée","ref":"9b16ccef-9a3b-4014-8e15-e9ecc33b8a6f","success":true} e2e-dmod-c1|3580|1790|is_Closed]
+✓ B. Différé partiellement réglé : modification refusée, message explicite, aucune copie [{"msg":"Ce différé a déjà reçu un règlement (partiel ou total) : il ne peut plus être modifié.","code":"REFUS_MODIFICATION","success":false}]
+✓ B. La vente et sa dette restent intactes [e2e-dmod-c1|3580|1790|is_Closed]
+✓ B. Différé partiellement réglé : annulation refusée, message explicite [{"msg":"Ce différé a déjà reçu un règlement (partiel ou total) : il ne peut plus être annulé.","code":"ETAT","success":false}]
+✓ A. Vente différée modifiée puis payée au comptant : plus de dette pour cette vente sur le compte du client [{"msg":"Opération effectuée avec success","ref":"5d54a736-7c3f-46db-bfbe-a437dc5d702f","success":true,"copy":true} restes 3580 -&gt; 1790 copie e2e-dmod-c1|0|0|delete]
+✓ C. Vente modifiée recloturée en différé pour un autre client : la dette passe sur ce client [{"msg":"Opération effectuée avec success","ref":"da91a08d-790f-455b-b216-db1c31ba4aae","success":true,"copy":true} copie e2e-dmod-c2|1790|1790|is_Closed]
+✓ D. Clôture de la copie refusée (type de vente changé) : la vente d'origine n'est pas annulée [{"msg":"Désolé impossible de transformer une vente au comptant","success":false,"codeError":0} origine 0|is_Closed ligne e2e-dmod-c1|1790|1790|is_Closed]
+✓ D. Puis clôture correcte : l'origine est annulée, une seule dette [{"msg":"Opération effectuée avec success","ref":"3ae9f28a-7f68-4a4c-ba5c-28dda825c1fe","success":true,"copy":true}]
+✓ Cohérence e2e-dmod-c1 : solde du relevé = somme des restes dus [relevé 3580, restes 3580]
+✓ Cohérence e2e-dmod-c2 : solde du relevé = somme des restes dus [relevé 1790, restes 1790]
+✓ Aucune erreur JavaScript [[]]
+✓ Jeu d'essai retiré, stock remis</t>
+        </is>
+      </c>
+      <c r="E50" s="10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr"/>
+      <c r="G50" s="9" t="inlineStr"/>
       <c r="H50" s="9" t="inlineStr"/>
       <c r="I50" s="9" t="inlineStr"/>
       <c r="J50" s="9" t="inlineStr"/>
@@ -13242,22 +13251,30 @@
  - aucune erreur JavaScript, aucune fenetre du navigateur.</t>
         </is>
       </c>
-      <c r="D78" s="9" t="inlineStr"/>
-      <c r="E78" s="11" t="inlineStr">
-        <is>
-          <t>Échec</t>
-        </is>
-      </c>
-      <c r="F78" s="9" t="inlineStr">
-        <is>
-          <t>Test arrêté (code 1) avant la fin, sans contrôle en écart</t>
-        </is>
-      </c>
-      <c r="G78" s="9" t="inlineStr">
-        <is>
-          <t>Données d'essai : Clients d'essai restés en base après l'arrêt des serveurs à 11 h 07 (le test ne peut pas recréer son jeu d'essai) ; passait le matin. À rejouer après nettoyage.</t>
-        </is>
-      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>12 / 12 conformes
+✓ Précondition : fidélité active, client inscrit avec 200 points (1 000 FCFA), article de 3000 FCFA [{"msg":"Ajustement enregistré.","seuil":0,"valeur":1000,"success":true,"utilisable":true,"solde":200}]
+✓ Article ajouté : net à payer &gt; 1 000 FCFA [3000]
+✓ Client non inscrit : pas d'encadré des points [{"vue":false,"texte":"","actif":false}]
+✓ L'ancien chemin reste : mode « Points fidélité » proposé dans la liste [3,2,4,19,1,8,9,7,20,10]
+✓ Client inscrit associé : « 200 point(s) = 1 000 FCFA » et la case « Utiliser » active [{"vue":true,"texte":"★ 200 point(s) = 1.000 FCFA","actif":true}]
+✓ « Utiliser » coché : « Points fidélité » en second mode, 1 000 FCFA, verrouillé [{"mode":"20","vue":true,"valeur":1000,"libelle":"POINTS FIDÉLITÉ 🔒","verrou":true}]
+✓ Décoché : second mode retiré [{"mode":null,"vue":false,"valeur":null,"libelle":"","verrou":true}]
+✓ Recoché : de nouveau 1 000 FCFA en points [{"mode":"20","vue":true,"valeur":1000,"libelle":"POINTS FIDÉLITÉ 🔒","verrou":true}]
+✓ « Terminer la vente » : vente clôturée, espèces 2000 + Points fidélité 1 000 [is_Closed / 1:2000,20:1000]
+✓ 200 points débités au client
+✓ Aucune erreur JavaScript, aucune fenêtre du navigateur []
+✓ Jeu d'essai retiré, paramètres remis</t>
+        </is>
+      </c>
+      <c r="E78" s="10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="inlineStr"/>
+      <c r="G78" s="9" t="inlineStr"/>
       <c r="H78" s="9" t="inlineStr"/>
       <c r="I78" s="9" t="inlineStr"/>
       <c r="J78" s="9" t="inlineStr"/>
@@ -18517,22 +18534,43 @@
  - ecran de vente : avertissement immediat quand les points ne suffisent pas ; aucune erreur JavaScript.</t>
         </is>
       </c>
-      <c r="D164" s="9" t="inlineStr"/>
-      <c r="E164" s="11" t="inlineStr">
-        <is>
-          <t>Échec</t>
-        </is>
-      </c>
-      <c r="F164" s="9" t="inlineStr">
-        <is>
-          <t>Test arrêté (code 1) avant la fin, sans contrôle en écart</t>
-        </is>
-      </c>
-      <c r="G164" s="9" t="inlineStr">
-        <is>
-          <t>Données d'essai : Clients d'essai restés en base après l'arrêt des serveurs à 11 h 07 (le test ne peut pas recréer son jeu d'essai) ; passait le matin. À rejouer après nettoyage.</t>
-        </is>
-      </c>
+      <c r="D164" s="9" t="inlineStr">
+        <is>
+          <t>25 / 25 conformes
+✓ Fidélité désactivée : « Points fidélité » absent des modes de la caisse [["3","2","4","19","1","8","9","7","6","10"]]
+✓ Fidélité activée : « Points fidélité » proposé à la caisse [["3","2","4","19","1","8","9","7","20","6","10"]]
+✓ Précondition : le client a 200 points (1 000 FCFA) [{"msg":"Ajustement enregistré.","seuil":10,"valeur":1000,"success":true,"utilisable":true,"solde":200}]
+✓ Caisse : solde et montant payable du client (200 points, 1 000 FCFA) [{"msg":"","seuil":10,"success":true,"utilisable":true,"solde":200,"actif":true,"montantMax":1000,"inscrit":true,"valeurPoint":5}]
+✓ A. Vente payée entièrement en points : clôturée, 57 point(s) débités [{"msg":"Opération effectuée avec success","ref":"7bb35edc-e3f9-4c94-9ddb-08787b5088df","success":true,"copy":false} solde 143]
+✓ A. Règlement « Points fidélité » enregistré (vente_reglement et mouvement de caisse)
+✓ A. Utilisation de points rattachée à la vente, avec sa valeur
+✓ B. Espèces + points : seuls les 60 points du second mode sont débités [{"msg":"Opération effectuée avec success","ref":"0e03f956-b3fc-4ba9-af63-4024b8bacfc2","success":true,"copy":false} solde 83]
+✓ B. Deux règlements enregistrés : espèces et points
+✓ C. Points insuffisants : clôture refusée avec le solde du client [{"msg":"Paiement en points refusé : 2850 FCFA demandent 570 point(s), le client n'en a que 83 (415 FCFA).","success":false,"codeError":0}]
+✓ C. Vente non enregistrée : toujours en cours, stock et points inchangés
+✓ D. Sans client : refusée [{"msg":"Paiement en points : choisissez d'abord le client de la vente.","success":false,"codeError":0}]
+✓ D. Vente en dépôt payée en points : refusée [{"msg":"Le paiement en points fidélité n'est pas possible pour une vente en dépôt.","success":false}]
+✓ Points gagnés sur la seule part payée autrement qu'en points (A : 0, B : net − 300) [A 0 B 270]
+✓ Ticket Z : ligne « Points fidélité » [{"data":{"datas":[{"modePaymentAmounts":[{"modeLibelle":"Espèce(vno/vo)","montant":"270"},{"modeLibelle":"Points fidélité (vno/vo)","montant":"585"},{"modeLibelle":"Différé","montant":"300"}],"user":"]
+✓ Balance vente-caisse : colonne « Points fidélité » = 585 FCFA [{"fondCaisse":0,"montantRegleTp":0,"rationAV":0,"montantSortie":0,"montantEsp":270,"montantRemise":0,"nbreVente":2,"montantEntre":0,"marge":288,"montantNet":855,"panierMoyen":427,"montantPointsFidelite":585,"ratioVA":0,"montantVirement":0,"montantCheque":0,"pourcentage":0,"montantHT":855,"montantReg]
+✓ Recettes : colonne « Points fidélité » = 585 FCFA, hors solde [{"montantReglementFacture":0,"montantEspece":270,"montantHt":855,"nbreClient":2,"montantSolde":270,"montantSortie":0,"montantEcart":-270,"montantRemise":0,"montantMobile":0,"montantEntre":0,"montantCb":0,"montantNet":855,"detailMobile":{},"montantPointsFidelite":585,"montantVirement":0,"montantChequ]
+✓ Balance parapharmacie : champ « Points fidélité » présent [{"metaData":{"fondCaisse":0,"montantRegleTp":0,"rationAV":0,"montantSortie":0,"montantEsp":0,"montantRemise":0,"nbreVente":0,"montantEntre":0,"marge":0,"montantNet":0,"panierMoyen":0,"montantPointsFid]
+✓ Écran des recettes : colonne « Pts fidélité »
+✓ Écran de la balance : colonne et total « Pts fidélité »
+✓ Logo du mode « Points fidélité » (POINTSFIDELITE.png) chargé [128]
+✓ Annulation de la vente payée en points : 57 point(s) rendus au client [{"msg":"L'opération effectuée avec success","ref":"9a475145-d3d9-43e0-ad06-e10ab0375fb4","success":true} solde 83 -&gt; 140]
+✓ Écran de vente : avertissement quand les points ne couvrent pas le net (solde, montant payable, conseil espèces + points) [Le client a 140 point(s), soit 700 FCFA, pour un net de 50.000 FCFA.Pour payer le reste autrement : choisissez « Espèces », saisissez le montant reçu, puis « Points fidélité » comme second mode pour 700 FCFA au plus.]
+✓ Aucune erreur JavaScript
+✓ Jeu d'essai retiré, paramètres de fidélité et mode remis</t>
+        </is>
+      </c>
+      <c r="E164" s="10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F164" s="9" t="inlineStr"/>
+      <c r="G164" s="9" t="inlineStr"/>
       <c r="H164" s="9" t="inlineStr"/>
       <c r="I164" s="9" t="inlineStr"/>
       <c r="J164" s="9" t="inlineStr"/>

</xml_diff>

<commit_message>
Test des onglets du dépôt : rayons choisis parmi ceux qui portent des articles, dépôt d'essai retiré si la pose échoue
Le premier rayon de la base était vide : la pose échouait (« NULL » inséré comme article) et laissait le dépôt
« DEPOT E2E ONGLETS », que l'écran Vente dépôt choisissait ensuite dans le test du QR publicitaire. Rapport et cahier
de recette mis à jour (370 / 422).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/recette/CAHIER_RECETTE_COMPLET_2026-10-30.xlsx
+++ b/docs/recette/CAHIER_RECETTE_COMPLET_2026-10-30.xlsx
@@ -653,7 +653,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>422 tests joués par l'écran, 369 OK, 53 en échec. Chaque test a été joué seul, par le vrai chemin de l'écran, et retire ses données à la fin.</t>
+          <t>422 tests joués par l'écran, 370 OK, 52 en échec. Chaque test a été joué seul, par le vrai chemin de l'écran, et retire ses données à la fin.</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>SYNTHÈSE — 422 tests, 369 OK, 53 en échec selon Claude</t>
+          <t>SYNTHÈSE — 422 tests, 370 OK, 52 en échec selon Claude</t>
         </is>
       </c>
     </row>
@@ -3765,10 +3765,10 @@
         <v>12</v>
       </c>
       <c r="D21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21">
         <f>COUNTA('Journal'!$I$5:$I$16)</f>
@@ -4350,7 +4350,7 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>12 tests : 10 OK, 2 en échec selon Claude</t>
+          <t>12 tests : 11 OK, 1 en échec selon Claude</t>
         </is>
       </c>
     </row>
@@ -4701,38 +4701,29 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>11 / 13 conformes
+          <t>13 / 13 conformes
 ✓ Vente : lien scanné → aucun appel au serveur, « QR code publicitaire » sans fenêtre, champ vidé [{"champ":"","fenetre":false,"texte":true} appels : ]
-✓ Vente : un vrai code scanné ensuite est cherché normalement [http://localhost:8080/prestige/api/v1/vente/findone/0000105?_dc=1793370985067]
-✗ Vente dépôt : lien scanné → aucun appel au serveur, « QR code publicitaire » sans fenêtre, champ vidé [{"champ":"htt","fenetre":false,"texte":false} appels : ]
-✗ Vente dépôt : code avec « / » et « # » envoyé encodé []
+✓ Vente : un vrai code scanné ensuite est cherché normalement [http://localhost:8080/prestige/api/v1/vente/findone/0000105?_dc=1793374338742]
+✓ Vente dépôt : lien scanné → aucun appel au serveur, « QR code publicitaire » sans fenêtre, champ vidé [{"champ":"","fenetre":false,"texte":true} appels : ]
+✓ Vente dépôt : code avec « / » et « # » envoyé encodé [http://localhost:8080/prestige/api/v1/vente/findone/E2E%2F12%233?_dc=1793374351988]
 ✓ Proforma : lien scanné → aucun appel au serveur, « QR code publicitaire » sans fenêtre, champ vidé [{"champ":"","fenetre":false,"texte":true} appels : ]
-✓ Proforma : code avec « / » et « # » envoyé encodé [http://localhost:8080/prestige/api/v1/vente/findone/E2E%2F12%233?_dc=1793371007357]
+✓ Proforma : code avec « / » et « # » envoyé encodé [http://localhost:8080/prestige/api/v1/vente/findone/E2E%2F12%233?_dc=1793374365157]
 ✓ Ajustement : lien scanné → aucun appel au serveur, « QR code publicitaire » sans fenêtre, champ vidé [{"champ":"","fenetre":false,"texte":true} appels : ]
-✓ Ajustement : code avec « / » et « # » envoyé encodé [http://localhost:8080/prestige/api/v1/vente/findone/E2E%2F12%233?_dc=1793371019754]
+✓ Ajustement : code avec « / » et « # » envoyé encodé [http://localhost:8080/prestige/api/v1/vente/findone/E2E%2F12%233?_dc=1793374377458]
 ✓ Vente en dépôt (extensions) : lien scanné → aucun appel au serveur, « QR code publicitaire » sans fenêtre, champ vidé [{"champ":"","fenetre":false,"texte":true} appels : ]
-✓ Vente en dépôt (extensions) : code avec « / » et « # » envoyé encodé [http://localhost:8080/prestige/api/v1/vente/findone/E2E%2F12%233?_dc=1793371032832]
+✓ Vente en dépôt (extensions) : code avec « / » et « # » envoyé encodé [http://localhost:8080/prestige/api/v1/vente/findone/E2E%2F12%233?_dc=1793374390385]
 ✓ Aucune erreur JavaScript []
-✓ Aucun ajustement ni vente créé par l'essai [780/476288 → 780/476288]
+✓ Aucun ajustement ni vente créé par l'essai [780/476280 → 780/476280]
 ✓ Client et dépôt d'essai retirés</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>Échec</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Vente dépôt : lien scanné → aucun appel au serveur, « QR code publicitaire » sans fenêtre, champ vidé [{"champ":"htt","fenetre":false,"texte":false} appels : ]
-Vente dépôt : code avec « / » et « # » envoyé encodé []</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>À examiner : Partie « vente dépôt » en échec deux fois de suite l'après-midi (champ partiellement saisi) ; passait le matin.</t>
-        </is>
-      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="9" t="inlineStr"/>
       <c r="H10" s="9" t="inlineStr"/>
       <c r="I10" s="9" t="inlineStr"/>
       <c r="J10" s="9" t="inlineStr"/>
@@ -11395,7 +11386,70 @@
 Tout ce que le test pose est retiré à la fin.</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr"/>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>57 / 59 conformes
+✓ Précondition : des articles dans plusieurs rayons [[{"id":"1412637135705554382","pa":675,"pv":1020,"stock":10,"zone":"14122419543881965607"},{"id":"14127214948274638940","pa":912,"pv":1380,"stock":11,"zone":"14122419543881965607"},{"id":"14131942241735077180","pa":977,"pv":1500,"stock":20,"zone":"14510223537039359655"}]]
+✓ Le menu séparé « Vente du dépôt » a disparu : la vente vit dans l onglet
+✓ Son privilège est conservé : il garde son sens pour l onglet
+✓ Le menu est passé dans GESTION DES TIERS-PAYANTS [53251827585053722655|GESTION DES TIERS-PAYANTS]
+✓ Il garde son identifiant et son privilège : seule la rubrique a changé [20260917|P_SM_DEPOT_EXTENSION]
+✓ Les quatre onglets ont chacun leur privilège [P_DEPOT_EXT_CA=11 P_DEPOT_EXT_POINT_CAISSE=11 P_DEPOT_EXT_VALORISATION=11 P_VENTE_DEPOT_EXTENSION=12]
+✓ Qui ouvre l écran garde l onglet P_DEPOT_EXT_VALORISATION [0 rôle(s) privé(s) de cet onglet]
+✓ Qui ouvre l écran garde l onglet P_VENTE_DEPOT_EXTENSION [0 rôle(s) privé(s) de cet onglet]
+✓ Qui ouvre l écran garde l onglet P_DEPOT_EXT_CA [0 rôle(s) privé(s) de cet onglet]
+✓ Qui ouvre l écran garde l onglet P_DEPOT_EXT_POINT_CAISSE [0 rôle(s) privé(s) de cet onglet]
+✓ L écran s ouvre [ok]
+✓ Les quatre onglets sont là, la saisie de vente en premier [["Saisir vente dépôt","Valorisation","Chiffre d'affaires","Point de caisse"]]
+✓ L écran s ouvre donc sur la saisie de vente
+✓ Chaque onglet porte sa propre classe de couleur [["x-tab depot-onglet-vente x-unselectable x-box-item x-tab-default x-active x-tab-active x-tab-default-active x-top-active x-tab-top-active x-tab-default-top-active x-noicon x-tab-noicon x-tab-default-noicon x-top x-tab-top x-tab-default-top","x-tab depot-onglet-valorisation x-unselectable x-box-item x-tab-default x-noicon x-tab-noicon x-]
+✗ C est le fond de l onglet qui est coloré, et les quatre fonds sont différents [["rgb(30, 58, 95)","rgb(255, 255, 255)","rgb(255, 255, 255)","rgb(255, 255, 255)"]]
+✗ Le libellé reste blanc sur les quatre onglets [["rgb(255, 255, 255)","rgb(52, 73, 94)","rgb(52, 73, 94)","rgb(52, 73, 94)"]]
+✓ L onglet ouvert se distingue des onglets fermés (teinte pleine contre teinte claire) [{"ouvert":"rgb(30, 58, 95)","autres":["rgb(30, 58, 95)","rgb(255, 255, 255)","rgb(255, 255, 255)","rgb(255, 255, 255)"]}]
+✓ Le service dit, onglet par onglet, à quoi l opérateur a droit [{"pointCaisse":true,"success":true,"valorisation":true,"vente":true,"ca":true}]
+✓ Un seul sélecteur de dépôt pilote l écran
+✓ La saisie de vente garde son propre sélecteur (dépôt redemandé à chaque vente)
+✓ Le dépôt se choisit une fois en haut de l écran [E2E-ONG-DEPOT]
+✓ La vue simple liste les articles du dépôt
+✓ La bascule affiche bien la vue par emplacement [depotextensionemplacement]
+✓ La valorisation est ventilée par rayon, sur plusieurs lignes [[{"emplacement":"DETAILS","articles":1,"valeurAchat":19540,"valeurVente":30000},{"emplacement":"SIROPS RHUME ET GRIPPE","articles":2,"valeurAchat":16782,"valeurVente":25380}]]
+✓ La somme des lignes fait exactement le total du dépôt [somme achat=36322/36322 vente=55380/55380]
+✓ Le total du dépôt est rappelé sous la ventilation, pour pouvoir vérifier la somme [Total du dépôt — valeur d'achat 36.322 CFA, valeur de vente 55.380 CFA (la somme des lignes ci-dessus doit faire ce total)]
+✓ Le dépôt de l écran prérenseigne la saisie de vente
+✓ La saisie de vente est bien celle de l écran de vente dupliqué (tiers payants, avoirs, préventes)
+✓ Le dépôt de la vente est en lecture seule : il vient de l écran, il ne se saisit pas ici [{"titre":"VENTE EN DÉPÔT – VENTE AU COMPTANT – DEPOT E2E ONGLETS","valeur":"E2E-ONG-DEPOT","lectureSeule":true,"enErreur":false,"grise":true}]
+✓ Il porte le dépôt choisi en haut, et le titre le nomme [{"titre":"VENTE EN DÉPÔT – VENTE AU COMPTANT – DEPOT E2E ONGLETS","valeur":"E2E-ONG-DEPOT","lectureSeule":true,"enErreur":false,"grise":true}]
+✓ Il n est jamais en erreur : ce n est plus une saisie, c est un rappel
+✓ Après une vente validée, le dépôt en cours est CONSERVÉ et reste grisé [{"titre":"VENTE EN DÉPÔT – VENTE AU COMPTANT – DEPOT E2E ONGLETS","valeur":"E2E-ONG-DEPOT","lectureSeule":true,"enErreur":false,"grise":true}]
+✓ Et le titre nomme toujours le dépôt [VENTE EN DÉPÔT – VENTE AU COMPTANT – DEPOT E2E ONGLETS]
+✓ Sans dépôt choisi, le titre n en nomme aucun : il ne retarde jamais [{"titre":"VENTE EN DÉPÔT – VENTE AU COMPTANT","valeur":null,"lectureSeule":true,"enErreur":false,"grise":true}]
+✓ L onglet Chiffre d affaires propose une période et ne charge rien tout seul
+✓ La période part des dates DU JOUR [{"debut":"2026-10-30","fin":"2026-10-30","aujourdhui":"2026-10-30","imprimer":true}]
+✓ L impression reste inactive avant toute recherche : on n imprime pas une grille vide
+✓ Les colonnes sont celles demandées, dans l ordre demandé [["typeVente","montantTTC","montantNet","marge","nbreVente","montantEsp","montantTp"]]
+✓ La colonne « règlement » a disparu [["typeVente","montantTTC","montantNet","marge","nbreVente","montantEsp","montantTp"]]
+✓ Chaque colonne de montant porte son total [[{"texte":"TYPE DE VENTE","champ":"typeVente","somme":""},{"texte":"MONTANT TTC","champ":"montantTTC","somme":"sum"},{"texte":"MONTANT NET","champ":"montantNet","somme":"sum"},{"texte":"MARGE","champ":"marge","somme":"sum"},{"texte":"NBRE VENTES","champ":"nbreVente","somme":"sum"},{"texte":"MONTANT ESPÈCES","champ":"montantEsp","somme":"s]
+✓ Le chiffre d affaires du dépôt répond et nomme le dépôt [{"totaux":"DEPOT E2E ONGLETS — 0 vente(s) — net 0 CFA (TTC 0, marge 0, tiers payant 0)","lignes":0}]
+✓ Le rappel explique où est l argent : caisse de l officine, chiffre au dépôt
+✓ Une ligne TOTAL est affichée sous les lignes [{"lignes":0,"sommeNet":0,"pied":"TOTAL000000","piedChiffres":"000000"}]
+✓ Le total du net est bien la somme des lignes [{"lignes":0,"sommeNet":0,"pied":"TOTAL000000","piedChiffres":"000000"}]
+✓ L impression devient active après la recherche
+✓ Le chiffre d affaires s imprime, servi en flux dans l onglet [{"statut":200,"type":"application/pdf","disposition":"inline; filename=\"chiffre_affaires_depot.pdf\""}]
+✓ Le document est un vrai PDF
+✓ Sans vente sur la période, l édition le dit au lieu de rendre une page vide [() (PHARMACIE DE LA CAPITALE) (Ce dépôt n'a enregistré aucune vente sur la période demandée.)]
+✓ L édition du chiffre d affaires refuse l officine
+✓ L onglet Point de caisse embarque l écran existant, rendu et fonctionnel [{"rendu":true,"grille":true}]
+✓ Il porte les colonnes de l écran Point Caisse Dépôt, sans recopie [["Date/Période","Dépôt","Caissière","Montant Net","Espèces","Crédit"]]
+✓ Le dépôt choisi en haut de l écran est imposé au point de caisse [E2E-ONG-DEPOT]
+✓ Sans le privilège, le service ne propose plus cet onglet [{"pointCaisse":true,"success":true,"valorisation":true,"vente":true,"ca":false}]
+✓ L onglet est retiré de l écran, pas seulement grisé [{"onglets":["ongletVente","ongletValorisation","ongletPointCaisse"],"actif":"ongletVente"}]
+✓ L écran reste utilisable et s ouvre sur un onglet existant [{"onglets":["ongletVente","ongletValorisation","ongletPointCaisse"],"actif":"ongletVente"}]
+✓ Et le service refuse les données, même appelé directement [{"total":0,"success":false,"message":"Votre profil ne donne pas accès à cette partie de l'écran."}]
+✓ L édition est refusée elle aussi [403]
+✓ Le privilège est rendu à la fin du contrôle
+✓ Aucune erreur JavaScript pendant tout le parcours</t>
+        </is>
+      </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
           <t>Échec</t>
@@ -11403,12 +11457,13 @@
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>Test arrêté (code 1) avant la fin, sans contrôle en écart</t>
+          <t>C est le fond de l onglet qui est coloré, et les quatre fonds sont différents [["rgb(30, 58, 95)","rgb(255, 255, 255)","rgb(255, 255, 255)","rgb(255, 255, 255)"]]
+Le libellé reste blanc sur les quatre onglets [["rgb(255, 255, 255)","rgb(52, 73, 94)","rgb(52, 73, 94)","rgb(52, 73, 94)"]]</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
         <is>
-          <t>À examiner : Pas encore étudié : test à adapter à la copie ou défaut à confirmer.</t>
+          <t>À examiner : Le test va maintenant au bout (57 / 59) : seules les couleurs des onglets diffèrent (fond coloré sur le seul onglet actif, libellé non blanc sur les autres). Avant, il échouait dès la pose du jeu d'essai (rayon vide) et laissait son dépôt dans la base.</t>
         </is>
       </c>
       <c r="H47" s="9" t="inlineStr"/>

</xml_diff>